<commit_message>
Replaced url with uri in all external_reference columns
</commit_message>
<xml_diff>
--- a/obspy/io/sitexml/tests/data/sera_site_all.xlsx
+++ b/obspy/io/sitexml/tests/data/sera_site_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiriaki/Desktop/ITSAK/ORFEUS/SITEXML/obspy15/obspy/obspy/io/sitexml/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E2BF8C0-0499-D14C-BFC1-B66191B37BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520CE546-C154-2D42-B106-DCEFE96D6795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17320" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="siteOwner" sheetId="4" r:id="rId1"/>
@@ -138,9 +138,6 @@
     <t>siteClassEC8_description</t>
   </si>
   <si>
-    <t>siteClassEC8_url</t>
-  </si>
-  <si>
     <t>bedrockDepth_value</t>
   </si>
   <si>
@@ -171,9 +168,6 @@
     <t>bedrockDepth_description</t>
   </si>
   <si>
-    <t>bedrockDepth_url</t>
-  </si>
-  <si>
     <t>h800_value</t>
   </si>
   <si>
@@ -204,9 +198,6 @@
     <t>h800_description</t>
   </si>
   <si>
-    <t>h800_url</t>
-  </si>
-  <si>
     <t>geologicalUnit_value</t>
   </si>
   <si>
@@ -240,9 +231,6 @@
     <t>geologicalUnit_description</t>
   </si>
   <si>
-    <t>geologicalUnit_url</t>
-  </si>
-  <si>
     <t>siteMorphology</t>
   </si>
   <si>
@@ -360,9 +348,6 @@
     <t>resonanceFrequency_description</t>
   </si>
   <si>
-    <t>resonanceFrequency_url</t>
-  </si>
-  <si>
     <t>velocityS30_value</t>
   </si>
   <si>
@@ -408,9 +393,6 @@
     <t>velocityS30_description</t>
   </si>
   <si>
-    <t>velocityS30_url</t>
-  </si>
-  <si>
     <t>velocityProfileCount</t>
   </si>
   <si>
@@ -450,9 +432,6 @@
     <t>velocityProfile_description</t>
   </si>
   <si>
-    <t>velocityProfile_url</t>
-  </si>
-  <si>
     <t>0.7</t>
   </si>
   <si>
@@ -622,6 +601,27 @@
   </si>
   <si>
     <t>1:50000</t>
+  </si>
+  <si>
+    <t>siteClassEC8_uri</t>
+  </si>
+  <si>
+    <t>bedrockDepth_uri</t>
+  </si>
+  <si>
+    <t>h800_uri</t>
+  </si>
+  <si>
+    <t>geologicalUnit_uri</t>
+  </si>
+  <si>
+    <t>resonanceFrequency_uri</t>
+  </si>
+  <si>
+    <t>velocityS30_uri</t>
+  </si>
+  <si>
+    <t>velocityProfile_uri</t>
   </si>
 </sst>
 </file>
@@ -2106,61 +2106,61 @@
     </row>
     <row r="2" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>177</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>178</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>163</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>167</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>168</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="H2" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="I2" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="B2" s="24" t="s">
-        <v>184</v>
-      </c>
-      <c r="C2" s="25" t="s">
-        <v>185</v>
-      </c>
-      <c r="D2" s="25" t="s">
+      <c r="J2" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="E2" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="F2" s="25" t="s">
-        <v>175</v>
-      </c>
-      <c r="G2" s="26" t="s">
+      <c r="K2" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="L2" s="27" t="s">
+        <v>171</v>
+      </c>
+      <c r="M2" s="25" t="s">
+        <v>152</v>
+      </c>
+      <c r="N2" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="O2" s="25" t="s">
         <v>173</v>
-      </c>
-      <c r="H2" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="J2" s="25" t="s">
-        <v>177</v>
-      </c>
-      <c r="K2" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="L2" s="27" t="s">
-        <v>178</v>
-      </c>
-      <c r="M2" s="25" t="s">
-        <v>159</v>
-      </c>
-      <c r="N2" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="O2" s="25" t="s">
-        <v>180</v>
       </c>
       <c r="P2" s="28">
         <v>12345</v>
       </c>
       <c r="Q2" s="25" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="R2" s="25" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="S2" s="25" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="T2" s="25" t="s">
         <v>20</v>
@@ -2222,7 +2222,7 @@
         <v>29</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>30</v>
@@ -2249,153 +2249,153 @@
         <v>37</v>
       </c>
       <c r="S1" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="T1" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="U1" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="V1" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="W1" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="V1" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="W1" s="9" t="s">
+      <c r="X1" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="Y1" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Z1" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="AA1" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="AA1" s="9" t="s">
+      <c r="AB1" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="AB1" s="9" t="s">
+      <c r="AC1" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="AC1" s="9" t="s">
+      <c r="AD1" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="AF1" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="AE1" s="9" t="s">
+      <c r="AG1" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="AF1" s="9" t="s">
+      <c r="AH1" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="AI1" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="AG1" s="9" t="s">
+      <c r="AJ1" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="AH1" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="AI1" s="9" t="s">
+      <c r="AK1" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="AJ1" s="9" t="s">
+      <c r="AL1" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="AK1" s="9" t="s">
+      <c r="AM1" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="AL1" s="9" t="s">
+      <c r="AN1" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="AM1" s="9" t="s">
+      <c r="AO1" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="AN1" s="9" t="s">
+      <c r="AP1" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="AO1" s="9" t="s">
+      <c r="AQ1" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="AR1" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="AP1" s="9" t="s">
+      <c r="AS1" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="AT1" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="AQ1" s="9" t="s">
+      <c r="AU1" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="AR1" s="9" t="s">
+      <c r="AV1" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="AS1" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="AT1" s="9" t="s">
+      <c r="AW1" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="AU1" s="9" t="s">
+      <c r="AX1" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="AV1" s="9" t="s">
+      <c r="AY1" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="AW1" s="9" t="s">
+      <c r="AZ1" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="AX1" s="9" t="s">
+      <c r="BA1" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="AY1" s="9" t="s">
+      <c r="BB1" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="AZ1" s="9" t="s">
+      <c r="BC1" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="BA1" s="9" t="s">
+      <c r="BD1" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="BE1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="BB1" s="9" t="s">
+      <c r="BF1" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="BC1" s="9" t="s">
+      <c r="BG1" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="BD1" s="9" t="s">
+      <c r="BH1" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="BE1" s="9" t="s">
+      <c r="BI1" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="BF1" s="9" t="s">
+      <c r="BJ1" s="9" t="s">
         <v>74</v>
-      </c>
-      <c r="BG1" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="BH1" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="BI1" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="BJ1" s="9" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:62" ht="128.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="11" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F2" s="12">
         <v>239</v>
@@ -2403,37 +2403,37 @@
       <c r="G2" s="12"/>
       <c r="H2" s="12"/>
       <c r="I2" s="11" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="J2" s="12">
         <v>1</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="M2" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="N2" s="11">
         <v>2018</v>
       </c>
       <c r="O2" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="P2" s="17" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="Q2" s="11" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="R2" s="11" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="S2" s="17" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="T2" s="12">
         <v>40</v>
@@ -2442,34 +2442,34 @@
         <v>6</v>
       </c>
       <c r="V2" s="11" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="W2" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="X2" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="Y2" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="Z2" s="11">
         <v>2018</v>
       </c>
       <c r="AA2" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="AB2" s="17" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AC2" s="11" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AD2" s="11" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AE2" s="17" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="AF2" s="12">
         <v>10</v>
@@ -2478,104 +2478,104 @@
         <v>1</v>
       </c>
       <c r="AH2" s="17" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="AI2" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="AJ2" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AK2" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="AL2" s="11">
         <v>2018</v>
       </c>
       <c r="AM2" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="AN2" s="17" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AO2" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AP2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AQ2" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="AR2" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="AP2" s="11" t="s">
+      <c r="AS2" s="11" t="s">
         <v>83</v>
-      </c>
-      <c r="AQ2" s="17" t="s">
-        <v>191</v>
-      </c>
-      <c r="AR2" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="AS2" s="11" t="s">
-        <v>87</v>
       </c>
       <c r="AT2" s="13"/>
       <c r="AU2" s="13"/>
       <c r="AV2" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="AW2" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AX2" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="AY2" s="11">
         <v>2018</v>
       </c>
       <c r="AZ2" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="BA2" s="17" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="BB2" s="11" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="BC2" s="11" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="BD2" s="17" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="BE2" s="11" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="BF2" s="11" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="BG2" s="11" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="BH2" s="11" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="BI2" s="11" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="BJ2" s="17" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:62" ht="44" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="14" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F3" s="15">
         <v>120</v>
@@ -2583,35 +2583,35 @@
       <c r="G3" s="15"/>
       <c r="H3" s="15"/>
       <c r="I3" s="20" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="J3" s="15">
         <v>1</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="L3" s="20" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="M3" s="21" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="N3" s="11">
         <v>2023</v>
       </c>
       <c r="O3" s="21" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="P3" s="21" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="Q3" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="R3" s="15"/>
       <c r="S3" s="14" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="T3" s="16">
         <v>820</v>
@@ -2621,29 +2621,29 @@
         <v>0.8</v>
       </c>
       <c r="W3" s="17" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="X3" s="20" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="Y3" s="21" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="Z3" s="11">
         <v>2023</v>
       </c>
       <c r="AA3" s="21" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="AB3" s="21" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AC3" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AD3" s="15"/>
       <c r="AE3" s="14" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="AF3" s="16">
         <v>180</v>
@@ -2651,43 +2651,43 @@
       <c r="AG3" s="15"/>
       <c r="AH3" s="15"/>
       <c r="AI3" s="17" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="AJ3" s="20" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="AK3" s="21" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="AL3" s="11">
         <v>2023</v>
       </c>
       <c r="AM3" s="21" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="AN3" s="21" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AO3" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AP3" s="15"/>
       <c r="AQ3" s="14" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="AR3" s="14" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="AS3" s="15"/>
       <c r="AT3" s="32" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="AU3" s="15"/>
       <c r="AV3" s="14" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="AW3" s="14" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="AX3" s="15"/>
       <c r="AY3" s="11"/>
@@ -2701,10 +2701,10 @@
       <c r="BG3" s="15"/>
       <c r="BH3" s="15"/>
       <c r="BI3" s="14" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="BJ3" s="20" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -2744,190 +2744,190 @@
         <v>22</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="R1" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="U1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="V1" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AF1" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AG1" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="AH1" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AI1" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="AE1" s="2" t="s">
+      <c r="AK1" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="AF1" s="2" t="s">
+      <c r="AL1" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="AG1" s="2" t="s">
+      <c r="AM1" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AN1" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="AI1" s="2" t="s">
+      <c r="AO1" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="AJ1" s="2" t="s">
+      <c r="AP1" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="AL1" s="2" t="s">
+      <c r="AR1" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="AM1" s="2" t="s">
+      <c r="AS1" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="AN1" s="2" t="s">
+      <c r="AT1" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="AO1" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="AP1" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="AQ1" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="AR1" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="AS1" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="AT1" s="2" t="s">
-        <v>141</v>
-      </c>
       <c r="AU1" s="2" t="s">
-        <v>142</v>
+        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:47" ht="128.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5">
         <v>0.8</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="L2" s="11">
         <v>2018</v>
       </c>
       <c r="M2" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="Q2" s="18" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="R2" s="4">
         <v>620</v>
@@ -2939,43 +2939,43 @@
         <v>0.5</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="X2" s="4">
         <v>1</v>
       </c>
       <c r="Y2" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="Z2" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AA2" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="AB2" s="11">
         <v>2018</v>
       </c>
       <c r="AC2" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="AD2" s="18" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AE2" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AF2" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AG2" s="18" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="AH2" s="4">
         <v>33</v>
@@ -2993,82 +2993,82 @@
         <v>1</v>
       </c>
       <c r="AM2" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="AN2" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AO2" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="AP2" s="11">
         <v>2018</v>
       </c>
       <c r="AQ2" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="AR2" s="18" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AT2" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AU2" s="18" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:47" ht="128" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="6" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="7">
         <v>1</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="I3" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="J3" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="K3" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="L3" s="11">
         <v>2018</v>
       </c>
       <c r="M3" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="Q3" s="18" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="R3" s="8">
         <v>620</v>
@@ -3080,43 +3080,43 @@
         <v>0.7</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="V3" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="W3" s="6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="X3" s="8">
         <v>1</v>
       </c>
       <c r="Y3" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="Z3" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AA3" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="AB3" s="11">
         <v>2018</v>
       </c>
       <c r="AC3" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="AD3" s="19" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AE3" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AF3" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AG3" s="19" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="AH3" s="8">
         <v>33</v>
@@ -3134,82 +3134,82 @@
         <v>1</v>
       </c>
       <c r="AM3" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="AN3" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AO3" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="AP3" s="11">
         <v>2018</v>
       </c>
       <c r="AQ3" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="AR3" s="19" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AS3" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AT3" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AU3" s="19" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" spans="1:47" ht="128" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>167</v>
-      </c>
       <c r="D4" s="6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7">
         <v>0.5</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="J4" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="K4" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="L4" s="11">
         <v>2018</v>
       </c>
       <c r="M4" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="Q4" s="18" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="R4" s="8">
         <v>620</v>
@@ -3221,43 +3221,43 @@
         <v>0.8</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="V4" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="W4" s="6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="X4" s="8">
         <v>1</v>
       </c>
       <c r="Y4" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="Z4" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AA4" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="AB4" s="11">
         <v>2018</v>
       </c>
       <c r="AC4" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="AD4" s="19" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AE4" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AF4" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AG4" s="19" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="AH4" s="8">
         <v>33</v>
@@ -3275,78 +3275,78 @@
         <v>1</v>
       </c>
       <c r="AM4" s="17" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="AN4" s="17" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="AO4" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="AP4" s="11">
         <v>2018</v>
       </c>
       <c r="AQ4" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="AR4" s="19" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AS4" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AT4" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="AU4" s="19" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:47" ht="44" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="6" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7">
         <v>0.6</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="H5" s="7"/>
       <c r="I5" s="17" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="J5" s="20" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="K5" s="21" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="L5" s="11">
         <v>2023</v>
       </c>
       <c r="M5" s="21" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="N5" s="21" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="O5" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="P5" s="15"/>
       <c r="Q5" s="20" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="R5" s="8">
         <v>497</v>
@@ -3356,37 +3356,37 @@
         <v>0.8</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="V5" s="7"/>
       <c r="W5" s="7"/>
       <c r="X5" s="6" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="Y5" s="17" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="Z5" s="20" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="AA5" s="21" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="AB5" s="11">
         <v>2023</v>
       </c>
       <c r="AC5" s="21" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="AD5" s="21" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="AE5" s="20" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="AF5" s="15"/>
       <c r="AG5" s="20" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>

</xml_diff>

<commit_message>
Enforced NET.STA notation in station_code (schema and API)
</commit_message>
<xml_diff>
--- a/obspy/io/sitexml/tests/data/sera_site_all.xlsx
+++ b/obspy/io/sitexml/tests/data/sera_site_all.xlsx
@@ -1985,7 +1985,7 @@
       </c>
       <c r="C2" s="18" t="inlineStr">
         <is>
-          <t>ABCD</t>
+          <t>XX.ABCD</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -2261,7 +2261,7 @@
       </c>
       <c r="C3" s="20" t="inlineStr">
         <is>
-          <t>ZWXY</t>
+          <t>YY.ZWXY</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Updated topography/morphology values for consistency
</commit_message>
<xml_diff>
--- a/obspy/io/sitexml/tests/data/sera_site_all.xlsx
+++ b/obspy/io/sitexml/tests/data/sera_site_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiriaki/Desktop/ITSAK/ORFEUS/SITEXML/obspy15/obspy/obspy/io/sitexml/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3741101E-469E-1848-B822-BFA4BBFABB77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A643376-EB79-0248-8AC2-0EF7580E5894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17320" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="siteOwner" sheetId="1" r:id="rId1"/>
@@ -580,9 +580,6 @@
     <t>0.25</t>
   </si>
   <si>
-    <t>Slope</t>
-  </si>
-  <si>
     <t>T1</t>
   </si>
   <si>
@@ -737,6 +734,9 @@
   </si>
   <si>
     <t>0</t>
+  </si>
+  <si>
+    <t>Valley - Basin</t>
   </si>
 </sst>
 </file>
@@ -2617,23 +2617,23 @@
       <c r="BD2" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="BE2" s="2" t="s">
+      <c r="BE2" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="BF2" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="BF2" s="2" t="s">
+      <c r="BG2" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="BG2" s="2" t="s">
+      <c r="BH2" s="2" t="s">
         <v>187</v>
-      </c>
-      <c r="BH2" s="2" t="s">
-        <v>188</v>
       </c>
       <c r="BI2" s="2" t="s">
         <v>48</v>
       </c>
       <c r="BJ2" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:62" ht="44" customHeight="1" x14ac:dyDescent="0.15">
@@ -2644,13 +2644,13 @@
         <v>67</v>
       </c>
       <c r="C3" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>191</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>192</v>
       </c>
       <c r="F3" s="5">
         <v>120</v>
@@ -2658,7 +2658,7 @@
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J3" s="5">
         <v>1</v>
@@ -2751,18 +2751,18 @@
         <v>75</v>
       </c>
       <c r="AR3" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AS3" s="5"/>
       <c r="AT3" s="19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AU3" s="5"/>
       <c r="AV3" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="AW3" s="4" t="s">
         <v>196</v>
-      </c>
-      <c r="AW3" s="4" t="s">
-        <v>197</v>
       </c>
       <c r="AX3" s="5"/>
       <c r="AY3" s="2"/>
@@ -2779,7 +2779,7 @@
         <v>68</v>
       </c>
       <c r="BJ3" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>
@@ -3483,103 +3483,103 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C1" t="s">
         <v>199</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>200</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>201</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>202</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>203</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>204</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>205</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>206</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>207</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>208</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>209</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>210</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>211</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>212</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>213</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>214</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>215</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>216</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>217</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>218</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>219</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>220</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>221</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>222</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>223</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>224</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>225</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>226</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>227</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AF1" t="s">
         <v>228</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AG1" t="s">
         <v>229</v>
       </c>
-      <c r="AG1" t="s">
+      <c r="AH1" t="s">
         <v>230</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="42" x14ac:dyDescent="0.15">
@@ -3587,61 +3587,61 @@
         <v>46</v>
       </c>
       <c r="B2" t="s">
+        <v>231</v>
+      </c>
+      <c r="C2" t="s">
         <v>232</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>233</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>234</v>
       </c>
-      <c r="E2" t="s">
-        <v>235</v>
-      </c>
       <c r="F2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K2" s="18"/>
       <c r="M2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="O2" s="18"/>
       <c r="Q2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="S2" s="18"/>
       <c r="U2" t="s">
+        <v>234</v>
+      </c>
+      <c r="V2" t="s">
+        <v>231</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>234</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>231</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>234</v>
+      </c>
+      <c r="AD2" t="s">
         <v>235</v>
       </c>
-      <c r="V2" t="s">
-        <v>232</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>235</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>232</v>
-      </c>
-      <c r="AC2" t="s">
-        <v>235</v>
-      </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>236</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>237</v>
       </c>
       <c r="AH2">
         <v>1</v>
@@ -3652,64 +3652,64 @@
         <v>66</v>
       </c>
       <c r="B3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C3" t="s">
         <v>232</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>233</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>234</v>
       </c>
-      <c r="E3" t="s">
-        <v>235</v>
-      </c>
       <c r="F3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H3" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="I3" t="s">
         <v>234</v>
       </c>
-      <c r="I3" t="s">
-        <v>235</v>
-      </c>
       <c r="J3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K3" s="18"/>
       <c r="L3" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="M3" t="s">
         <v>234</v>
       </c>
-      <c r="M3" t="s">
-        <v>235</v>
-      </c>
       <c r="N3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="O3" s="18"/>
       <c r="P3" s="18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="S3" s="18"/>
       <c r="T3" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="U3" t="s">
         <v>234</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
+        <v>231</v>
+      </c>
+      <c r="X3" s="18" t="s">
+        <v>233</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>234</v>
+      </c>
+      <c r="AD3" t="s">
         <v>235</v>
-      </c>
-      <c r="V3" t="s">
-        <v>232</v>
-      </c>
-      <c r="X3" s="18" t="s">
-        <v>234</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>235</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>236</v>
       </c>
       <c r="AH3">
         <v>1</v>

</xml_diff>

<commit_message>
Aligning velocity profile specific schema element/type names with API class/argument names.
</commit_message>
<xml_diff>
--- a/obspy/io/sitexml/tests/data/sera_site_all.xlsx
+++ b/obspy/io/sitexml/tests/data/sera_site_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiriaki/Desktop/ITSAK/ORFEUS/SITEXML/obspy15/obspy/obspy/io/sitexml/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A643376-EB79-0248-8AC2-0EF7580E5894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033C7510-F636-3543-94C8-0C2375E83EA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17320" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="siteOwner" sheetId="1" r:id="rId1"/>
@@ -133,36 +133,6 @@
     <t>boreholeLogsCount</t>
   </si>
   <si>
-    <t>velocityProfileQindex1</t>
-  </si>
-  <si>
-    <t>velocityProfile_title</t>
-  </si>
-  <si>
-    <t>velocityProfile_firstAuthor</t>
-  </si>
-  <si>
-    <t>velocityProfile_secondaryAuthors</t>
-  </si>
-  <si>
-    <t>velocityProfile_year</t>
-  </si>
-  <si>
-    <t>velocityProfile_booktitle</t>
-  </si>
-  <si>
-    <t>velocityProfile_language</t>
-  </si>
-  <si>
-    <t>velocityProfile_doi</t>
-  </si>
-  <si>
-    <t>velocityProfile_description</t>
-  </si>
-  <si>
-    <t>velocityProfile_uri</t>
-  </si>
-  <si>
     <t>quakeml:domain.ab/site/001</t>
   </si>
   <si>
@@ -691,18 +661,6 @@
     <t>velocityS30_report</t>
   </si>
   <si>
-    <t>velocityProfile_method</t>
-  </si>
-  <si>
-    <t>velocityProfile_evaluation</t>
-  </si>
-  <si>
-    <t>velocityProfile_reliability</t>
-  </si>
-  <si>
-    <t>velocityProfile_report</t>
-  </si>
-  <si>
     <t>f0_vs30</t>
   </si>
   <si>
@@ -737,6 +695,48 @@
   </si>
   <si>
     <t>Valley - Basin</t>
+  </si>
+  <si>
+    <t>velocityProfileSetQindex1</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_title</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_firstAuthor</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_secondaryAuthors</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_year</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_booktitle</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_language</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_doi</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_description</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_uri</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_evaluation</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_reliability</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_report</t>
+  </si>
+  <si>
+    <t>velocityProfileSet_method</t>
   </si>
 </sst>
 </file>
@@ -2120,126 +2120,126 @@
   <sheetData>
     <row r="1" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="L1" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="M1" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="N1" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="O1" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="P1" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="Q1" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="R1" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="S1" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="T1" s="10" t="s">
         <v>87</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="L1" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="M1" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="O1" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="P1" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q1" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="R1" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="S1" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="T1" s="10" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="L2" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="M2" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="N2" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="O2" s="13" t="s">
         <v>102</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="J2" s="13" t="s">
-        <v>107</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="M2" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="N2" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="O2" s="13" t="s">
-        <v>112</v>
       </c>
       <c r="P2" s="16">
         <v>12345</v>
       </c>
       <c r="Q2" s="13" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="R2" s="13" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="S2" s="13" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="T2" s="13" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2276,201 +2276,201 @@
         <v>1</v>
       </c>
       <c r="C1" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="N1" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="P1" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="Q1" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="R1" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="S1" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="T1" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="U1" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="V1" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="W1" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="Z1" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="AB1" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="AC1" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="T1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="U1" s="6" t="s">
+      <c r="AE1" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="V1" s="6" t="s">
+      <c r="AF1" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="AG1" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="AH1" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="AI1" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="Z1" s="6" t="s">
+      <c r="AJ1" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AK1" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="AB1" s="6" t="s">
+      <c r="AL1" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AM1" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="AD1" s="6" t="s">
+      <c r="AN1" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AO1" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="AF1" s="6" t="s">
+      <c r="AP1" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="AG1" s="6" t="s">
+      <c r="AQ1" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="AH1" s="6" t="s">
+      <c r="AR1" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="AI1" s="6" t="s">
+      <c r="AS1" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="AJ1" s="6" t="s">
+      <c r="AT1" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="AK1" s="6" t="s">
+      <c r="AU1" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="AL1" s="6" t="s">
+      <c r="AV1" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="AM1" s="6" t="s">
+      <c r="AW1" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="AN1" s="6" t="s">
+      <c r="AX1" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="AO1" s="6" t="s">
+      <c r="AY1" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="AP1" s="6" t="s">
+      <c r="AZ1" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="AQ1" s="6" t="s">
+      <c r="BA1" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="AR1" s="6" t="s">
+      <c r="BB1" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="AS1" s="6" t="s">
+      <c r="BC1" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="AT1" s="6" t="s">
+      <c r="BD1" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="AU1" s="6" t="s">
+      <c r="BE1" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="AV1" s="6" t="s">
+      <c r="BF1" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="AW1" s="6" t="s">
+      <c r="BG1" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="AX1" s="6" t="s">
+      <c r="BH1" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="AY1" s="6" t="s">
+      <c r="BI1" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="AZ1" s="6" t="s">
+      <c r="BJ1" s="6" t="s">
         <v>166</v>
-      </c>
-      <c r="BA1" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="BB1" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="BC1" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="BD1" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="BE1" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="BF1" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="BG1" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="BH1" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="BI1" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="BJ1" s="6" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="2" spans="1:62" ht="128.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="F2" s="3">
         <v>239</v>
@@ -2478,37 +2478,37 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="2" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="J2" s="3">
         <v>1</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="N2" s="2">
         <v>2018</v>
       </c>
       <c r="O2" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="P2" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="S2" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="T2" s="3">
         <v>40</v>
@@ -2517,34 +2517,34 @@
         <v>6</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="W2" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="X2" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="Y2" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="Z2" s="2">
         <v>2018</v>
       </c>
       <c r="AA2" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AB2" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AC2" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AD2" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AE2" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="AF2" s="3">
         <v>10</v>
@@ -2553,104 +2553,104 @@
         <v>1</v>
       </c>
       <c r="AH2" s="7" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="AI2" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="AJ2" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="AK2" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="AL2" s="2">
         <v>2018</v>
       </c>
       <c r="AM2" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AN2" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AO2" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AP2" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AQ2" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="AR2" s="2" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="AS2" s="2" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3"/>
       <c r="AV2" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="AW2" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="AX2" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="AY2" s="2">
         <v>2018</v>
       </c>
       <c r="AZ2" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="BA2" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="BB2" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="BC2" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="BD2" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="BE2" s="7" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
       <c r="BF2" s="2" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="BG2" s="2" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="BH2" s="2" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="BI2" s="2" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="BJ2" s="7" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:62" ht="44" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="4" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="F3" s="5">
         <v>120</v>
@@ -2658,35 +2658,35 @@
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
       <c r="I3" s="8" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="J3" s="5">
         <v>1</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="N3" s="2">
         <v>2023</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="P3" s="9" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="4" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="T3" s="5">
         <v>820</v>
@@ -2696,29 +2696,29 @@
         <v>0.8</v>
       </c>
       <c r="W3" s="7" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="X3" s="8" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="Y3" s="9" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="Z3" s="2">
         <v>2023</v>
       </c>
       <c r="AA3" s="9" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="AB3" s="9" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AC3" s="8" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="AD3" s="5"/>
       <c r="AE3" s="4" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="AF3" s="5">
         <v>180</v>
@@ -2726,43 +2726,43 @@
       <c r="AG3" s="5"/>
       <c r="AH3" s="5"/>
       <c r="AI3" s="7" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="AJ3" s="8" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="AK3" s="9" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="AL3" s="2">
         <v>2023</v>
       </c>
       <c r="AM3" s="9" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="AN3" s="9" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AO3" s="8" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="AP3" s="5"/>
       <c r="AQ3" s="4" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="AR3" s="4" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="AS3" s="5"/>
       <c r="AT3" s="19" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="AU3" s="5"/>
       <c r="AV3" s="4" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="AW3" s="4" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="AX3" s="5"/>
       <c r="AY3" s="2"/>
@@ -2776,10 +2776,10 @@
       <c r="BG3" s="5"/>
       <c r="BH3" s="5"/>
       <c r="BI3" s="4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="BJ3" s="8" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2920,85 +2920,85 @@
         <v>35</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>36</v>
+        <v>224</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>37</v>
+        <v>225</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>38</v>
+        <v>226</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>39</v>
+        <v>227</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>40</v>
+        <v>228</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>41</v>
+        <v>229</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>42</v>
+        <v>230</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>43</v>
+        <v>231</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>44</v>
+        <v>232</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>45</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:46" ht="128.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3">
         <v>0.8</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="L2" s="2">
         <v>2018</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="N2" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="Q2" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="R2" s="3">
         <v>620</v>
@@ -3010,43 +3010,43 @@
         <v>0.5</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="X2" s="3">
         <v>1</v>
       </c>
       <c r="Y2" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="Z2" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="AA2" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="AB2" s="2">
         <v>2018</v>
       </c>
       <c r="AC2" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AD2" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AE2" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AG2" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="AH2" s="3">
         <v>0</v>
@@ -3061,82 +3061,82 @@
         <v>1</v>
       </c>
       <c r="AL2" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="AM2" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="AN2" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="AO2" s="2">
         <v>2018</v>
       </c>
       <c r="AP2" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AQ2" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AR2" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AS2" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AT2" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:46" ht="128" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="4" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="5">
         <v>1</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="K3" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="L3" s="2">
         <v>2018</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="P3" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="Q3" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="R3" s="5">
         <v>620</v>
@@ -3148,43 +3148,43 @@
         <v>0.7</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="W3" s="4" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="X3" s="5">
         <v>1</v>
       </c>
       <c r="Y3" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="Z3" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="AA3" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="AB3" s="2">
         <v>2018</v>
       </c>
       <c r="AC3" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AD3" s="8" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AE3" s="4" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AF3" s="4" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AG3" s="8" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="AH3" s="5">
         <v>0</v>
@@ -3199,82 +3199,82 @@
         <v>1</v>
       </c>
       <c r="AL3" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="AM3" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="AN3" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="AO3" s="2">
         <v>2018</v>
       </c>
       <c r="AP3" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AQ3" s="8" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AR3" s="4" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AS3" s="4" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AT3" s="8" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:46" ht="128" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="4" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E4" s="5"/>
       <c r="F4" s="5">
         <v>0.5</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="L4" s="2">
         <v>2018</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="P4" s="2" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="Q4" s="7" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="R4" s="5">
         <v>620</v>
@@ -3286,43 +3286,43 @@
         <v>0.8</v>
       </c>
       <c r="U4" s="4" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="W4" s="4" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="X4" s="5">
         <v>1</v>
       </c>
       <c r="Y4" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="Z4" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="AA4" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="AB4" s="2">
         <v>2018</v>
       </c>
       <c r="AC4" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AD4" s="8" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AE4" s="4" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AF4" s="4" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AG4" s="8" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="AH4" s="5">
         <v>0</v>
@@ -3337,78 +3337,78 @@
         <v>1</v>
       </c>
       <c r="AL4" s="7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="AM4" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="AN4" s="7" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="AO4" s="2">
         <v>2018</v>
       </c>
       <c r="AP4" s="7" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="AQ4" s="8" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AR4" s="4" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="AS4" s="4" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="AT4" s="8" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:46" ht="44" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="4" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E5" s="5"/>
       <c r="F5" s="5">
         <v>0.6</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="7" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="L5" s="2">
         <v>2023</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="N5" s="9" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="P5" s="5"/>
       <c r="Q5" s="8" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="R5" s="5">
         <v>497</v>
@@ -3418,37 +3418,37 @@
         <v>0.8</v>
       </c>
       <c r="U5" s="4" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="V5" s="5"/>
       <c r="W5" s="5"/>
       <c r="X5" s="4" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="Y5" s="7" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="Z5" s="8" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="AA5" s="9" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="AB5" s="2">
         <v>2023</v>
       </c>
       <c r="AC5" s="9" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="AD5" s="9" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="AE5" s="8" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="AF5" s="5"/>
       <c r="AG5" s="8" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="AH5" s="5"/>
       <c r="AI5" s="5"/>
@@ -3483,165 +3483,165 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F1" t="s">
+        <v>192</v>
+      </c>
+      <c r="G1" t="s">
+        <v>193</v>
+      </c>
+      <c r="H1" t="s">
+        <v>194</v>
+      </c>
+      <c r="I1" t="s">
+        <v>195</v>
+      </c>
+      <c r="J1" t="s">
+        <v>196</v>
+      </c>
+      <c r="K1" t="s">
+        <v>197</v>
+      </c>
+      <c r="L1" t="s">
         <v>198</v>
       </c>
-      <c r="C1" t="s">
+      <c r="M1" t="s">
         <v>199</v>
       </c>
-      <c r="D1" t="s">
+      <c r="N1" t="s">
         <v>200</v>
       </c>
-      <c r="E1" t="s">
+      <c r="O1" t="s">
         <v>201</v>
       </c>
-      <c r="F1" t="s">
+      <c r="P1" t="s">
         <v>202</v>
       </c>
-      <c r="G1" t="s">
+      <c r="Q1" t="s">
         <v>203</v>
       </c>
-      <c r="H1" t="s">
+      <c r="R1" t="s">
         <v>204</v>
       </c>
-      <c r="I1" t="s">
+      <c r="S1" t="s">
         <v>205</v>
       </c>
-      <c r="J1" t="s">
+      <c r="T1" t="s">
         <v>206</v>
       </c>
-      <c r="K1" t="s">
+      <c r="U1" t="s">
         <v>207</v>
       </c>
-      <c r="L1" t="s">
+      <c r="V1" t="s">
         <v>208</v>
       </c>
-      <c r="M1" t="s">
+      <c r="W1" t="s">
         <v>209</v>
       </c>
-      <c r="N1" t="s">
+      <c r="X1" t="s">
         <v>210</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Y1" t="s">
         <v>211</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Z1" t="s">
+        <v>237</v>
+      </c>
+      <c r="AA1" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>235</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>236</v>
+      </c>
+      <c r="AD1" t="s">
         <v>212</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="AE1" t="s">
         <v>213</v>
       </c>
-      <c r="R1" t="s">
+      <c r="AF1" t="s">
         <v>214</v>
       </c>
-      <c r="S1" t="s">
+      <c r="AG1" t="s">
         <v>215</v>
       </c>
-      <c r="T1" t="s">
+      <c r="AH1" t="s">
         <v>216</v>
-      </c>
-      <c r="U1" t="s">
-        <v>217</v>
-      </c>
-      <c r="V1" t="s">
-        <v>218</v>
-      </c>
-      <c r="W1" t="s">
-        <v>219</v>
-      </c>
-      <c r="X1" t="s">
-        <v>220</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>221</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>222</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>223</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>224</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>225</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>226</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>227</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>228</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>229</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="42" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="C2" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="D2" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="E2" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="F2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="I2" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="J2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="K2" s="18"/>
       <c r="M2" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="N2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="O2" s="18"/>
       <c r="Q2" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="R2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="S2" s="18"/>
       <c r="U2" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="V2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="Y2" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="Z2" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="AC2" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="AD2" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="AE2" t="s">
-        <v>236</v>
+        <v>222</v>
       </c>
       <c r="AH2">
         <v>1</v>
@@ -3649,67 +3649,67 @@
     </row>
     <row r="3" spans="1:34" ht="42" x14ac:dyDescent="0.15">
       <c r="A3" s="18" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="C3" t="s">
-        <v>232</v>
+        <v>218</v>
       </c>
       <c r="D3" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="E3" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="F3" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="H3" s="18" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="I3" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="J3" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="K3" s="18"/>
       <c r="L3" s="18" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="M3" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="N3" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="O3" s="18"/>
       <c r="P3" s="18" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="R3" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="S3" s="18"/>
       <c r="T3" s="18" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="U3" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="V3" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
       <c r="X3" s="18" t="s">
-        <v>233</v>
+        <v>219</v>
       </c>
       <c r="Y3" t="s">
-        <v>234</v>
+        <v>220</v>
       </c>
       <c r="AD3" t="s">
-        <v>235</v>
+        <v>221</v>
       </c>
       <c r="AH3">
         <v>1</v>

</xml_diff>